<commit_message>
demo: the sample is synthetic at a real address; internal-only values are labelled; trade-out is gone; the upload form asks for the price per unit
Republished sample set (13 tabs, five downloads) from the restaged fixture: real demand,
supply, rent-comp and property-tax pulls for a real Tempe, AZ address around a fabricated
property; the ZIP-vs-metro home value and rent-to-income rows; two supply stages. Values the
internal pipeline produces that the demo deliberately does not read 'Internal pipeline
only' with the reason. The trade-out tab is removed from both pages (tabs.ts). The upload
form takes the purchase price per unit as a required field (band from /api/meta) and sends
it as price_per_unit. Page copy says what is real and what is fabricated.

Built clean (29 pages). Not pushed — push is the deploy.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/underwriting-demo/sample-rent-roll-analysis.xlsx
+++ b/public/downloads/underwriting-demo/sample-rent-roll-analysis.xlsx
@@ -9,8 +9,7 @@
   <sheets>
     <sheet name="Rent Roll" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Unit Mix Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lease Trade-Out" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Audit Trail" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Audit Trail" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -9367,222 +9366,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Lease trade-out</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Fixture Park — as of 2026-06-30</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Gross and effective are both stated: concessions are what separate them, and quoting one as the other is how a trade-out number becomes wrong.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n"/>
-      <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
-      <c r="D4" s="3" t="n"/>
-      <c r="E4" s="3" t="n"/>
-      <c r="F4" s="3" t="n"/>
-      <c r="G4" s="3" t="n"/>
-      <c r="H4" s="3" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Cohort</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>Leases</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>Prior rent</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>New rent (gross)</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Gross change ($)</t>
-        </is>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Gross change (%)</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>New rent (effective)</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>Effective change ($)</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>Effective change (%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="5" t="inlineStr">
-        <is>
-          <t>New</t>
-        </is>
-      </c>
-      <c r="B6" s="7" t="n">
-        <v>46</v>
-      </c>
-      <c r="C6" s="7" t="n">
-        <v>1706</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>1812</v>
-      </c>
-      <c r="E6" s="7">
-        <f>IFERROR(D6-C6,"")</f>
-        <v/>
-      </c>
-      <c r="F6" s="19">
-        <f>IFERROR((D6-C6)/C6,"")</f>
-        <v/>
-      </c>
-      <c r="G6" s="7" t="n">
-        <v>1774</v>
-      </c>
-      <c r="H6" s="7">
-        <f>IFERROR(G6-C6,"")</f>
-        <v/>
-      </c>
-      <c r="I6" s="19">
-        <f>IFERROR((G6-C6)/C6,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>Renewal</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="n">
-        <v>88</v>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>1698</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>1745</v>
-      </c>
-      <c r="E7" s="7">
-        <f>IFERROR(D7-C7,"")</f>
-        <v/>
-      </c>
-      <c r="F7" s="19">
-        <f>IFERROR((D7-C7)/C7,"")</f>
-        <v/>
-      </c>
-      <c r="G7" s="7" t="n">
-        <v>1745</v>
-      </c>
-      <c r="H7" s="7">
-        <f>IFERROR(G7-C7,"")</f>
-        <v/>
-      </c>
-      <c r="I7" s="19">
-        <f>IFERROR((G7-C7)/C7,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>First generation</t>
-        </is>
-      </c>
-      <c r="B8" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>1836</v>
-      </c>
-      <c r="E8" s="7">
-        <f>IFERROR(D8-C8,"")</f>
-        <v/>
-      </c>
-      <c r="F8" s="19">
-        <f>IFERROR((D8-C8)/C8,"")</f>
-        <v/>
-      </c>
-      <c r="G8" s="7" t="n">
-        <v>1790</v>
-      </c>
-      <c r="H8" s="7">
-        <f>IFERROR(G8-C8,"")</f>
-        <v/>
-      </c>
-      <c r="I8" s="19">
-        <f>IFERROR((G8-C8)/C8,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="9"/>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>A first-generation lease has no prior rent, so its percentage change is undefined and reads blank rather than as a number divided by zero.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9612,7 +9395,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>The rent roll, unit mix and trade-out. Every value below names the document it came from and where in it. A derived value names the values it was built from — one that could not would not have passed validation.</t>
+          <t>The rent roll and unit mix. Every value below names the document it came from and where in it. A derived value names the values it was built from — one that could not would not have passed validation.</t>
         </is>
       </c>
     </row>
@@ -9932,12 +9715,12 @@
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>3 entries</t>
+          <t>0 entries</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Synthetic lease trade-out report</t>
+          <t>Internal pipeline only</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -9953,7 +9736,7 @@
       <c r="F16" s="10" t="n"/>
       <c r="G16" s="23" t="inlineStr">
         <is>
-          <t>Cohort averages.</t>
+          <t>The internal pipeline reads a lease trade-out report (new versus renewal rents); the demo does not ask for one.</t>
         </is>
       </c>
     </row>

</xml_diff>